<commit_message>
Modify test cases and bug reports
</commit_message>
<xml_diff>
--- a/02_Manual_Testing/Test_Cases.xlsx
+++ b/02_Manual_Testing/Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\BookStack Demo WebTesting\BookStackDemo_WebTesting\02_Manual_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9DEA7D-2977-488A-8E38-210E66490157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2133069D-370A-4982-B92A-E04B49E20684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="236">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -466,9 +466,6 @@
     <t>Book creation fails and validation error is displayed.</t>
   </si>
   <si>
-    <t>Verify behavior when Name exceeds max length</t>
-  </si>
-  <si>
     <t>1. Enter Name of a book with 256 character length
 2. Enter Description 'Above Maximum Boundary (256)'
 3. Click 'Save Book'</t>
@@ -477,10 +474,6 @@
     <t>System should restrict input and display validation error.</t>
   </si>
   <si>
-    <t>Book Name: &lt;Name with 256 words&gt;
-Description: Above Maximum Boundary (256)</t>
-  </si>
-  <si>
     <t>1. Enter Name of a book already created
 2. Enter Description 'duplicate book names'
 3. Click 'Save Book'</t>
@@ -490,9 +483,6 @@
 Description: All things for the IT team</t>
   </si>
   <si>
-    <t>System accepts input.</t>
-  </si>
-  <si>
     <t>System restricts input and display validation error.</t>
   </si>
   <si>
@@ -517,16 +507,9 @@
     <t>Verify validity when creating books with the description field left blank</t>
   </si>
   <si>
-    <t>Verify behavior when Description exceeds max length</t>
-  </si>
-  <si>
     <t>1. Enter Name of a book
 2. Leave Description field blank
 3. Click 'Save Book'</t>
-  </si>
-  <si>
-    <t>Book Name: Fairy Tales
-Description: &lt;Description with 2000 words&gt;</t>
   </si>
   <si>
     <t>Book Name: Fairy Tales Story
@@ -807,16 +790,36 @@
     <t>System display 'Page Not Found' error page.</t>
   </si>
   <si>
-    <t>Verify behavior when Shelf exceeds max length</t>
-  </si>
-  <si>
     <t>1. Enter Name of a shelf with 256 character length
 2. Enter Description 'Above Maximum Boundary (256)'
 3. Click 'Save Shelf'</t>
   </si>
   <si>
-    <t>Shelf Name: &lt;Name with 256 words&gt;
+    <t>Verify behavior when Name exceeds max characters</t>
+  </si>
+  <si>
+    <t>Book Name: &lt;Name with 256 characters&gt;
 Description: Above Maximum Boundary (256)</t>
+  </si>
+  <si>
+    <t>Book Name: Fairy Tales
+Description: &lt;Description with 2000 characters&gt;</t>
+  </si>
+  <si>
+    <t>Verify behavior when Description exceeds max characters</t>
+  </si>
+  <si>
+    <t>Verify behavior when Shelf exceeds max characters</t>
+  </si>
+  <si>
+    <t>Shelf Name: &lt;Name with 256 characters&gt;
+Description: Above Maximum Boundary (256)</t>
+  </si>
+  <si>
+    <t>System accepts input in Shelf name.</t>
+  </si>
+  <si>
+    <t>System accepts input in Book name.</t>
   </si>
 </sst>
 </file>
@@ -1599,7 +1602,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>15</v>
@@ -1772,7 +1775,7 @@
         <v>129</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>130</v>
@@ -1804,7 +1807,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>27</v>
@@ -1839,7 +1842,7 @@
         <v>74</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>135</v>
+        <v>228</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>25</v>
@@ -1851,16 +1854,16 @@
         <v>27</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>137</v>
-      </c>
       <c r="I23" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>21</v>
@@ -1880,28 +1883,28 @@
         <v>75</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D24" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="F24" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>141</v>
+        <v>235</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>21</v>
@@ -1913,7 +1916,7 @@
         <v>97</v>
       </c>
       <c r="M24" s="8" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
@@ -1921,22 +1924,22 @@
         <v>76</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>25</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>130</v>
@@ -1962,7 +1965,7 @@
         <v>77</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>149</v>
+        <v>231</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>25</v>
@@ -1974,16 +1977,16 @@
         <v>27</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>151</v>
+        <v>230</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>21</v>
@@ -2012,19 +2015,19 @@
         <v>94</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>31</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>21</v>
@@ -2050,16 +2053,16 @@
         <v>25</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="H28" s="2" t="s">
         <v>100</v>
@@ -2085,7 +2088,7 @@
         <v>80</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>35</v>
@@ -2097,16 +2100,16 @@
         <v>36</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>13</v>
@@ -2126,13 +2129,13 @@
         <v>81</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>36</v>
@@ -2144,10 +2147,10 @@
         <v>38</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="J30" s="5" t="s">
         <v>13</v>
@@ -2179,16 +2182,16 @@
         <v>36</v>
       </c>
       <c r="F31" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="G31" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="H31" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>21</v>
@@ -2208,28 +2211,28 @@
         <v>83</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>141</v>
+        <v>234</v>
       </c>
       <c r="J32" s="5" t="s">
         <v>21</v>
@@ -2241,7 +2244,7 @@
         <v>97</v>
       </c>
       <c r="M32" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="86.4" x14ac:dyDescent="0.3">
@@ -2249,7 +2252,7 @@
         <v>84</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>35</v>
@@ -2258,19 +2261,19 @@
         <v>94</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J33" s="5" t="s">
         <v>13</v>
@@ -2296,22 +2299,22 @@
         <v>35</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="J34" s="5" t="s">
         <v>21</v>
@@ -2331,7 +2334,7 @@
         <v>86</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>35</v>
@@ -2340,19 +2343,19 @@
         <v>94</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>101</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>21</v>
@@ -2381,19 +2384,19 @@
         <v>94</v>
       </c>
       <c r="E36" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="F36" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>195</v>
-      </c>
       <c r="H36" s="2" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="J36" s="5" t="s">
         <v>13</v>
@@ -2419,13 +2422,13 @@
         <v>40</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>143</v>
+        <v>110</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>26</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>43</v>
@@ -2434,7 +2437,7 @@
         <v>102</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>32</v>
@@ -2463,19 +2466,19 @@
         <v>94</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="J38" s="5" t="s">
         <v>21</v>
@@ -2507,16 +2510,16 @@
         <v>26</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="J39" s="5" t="s">
         <v>21</v>
@@ -2536,28 +2539,28 @@
         <v>91</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>94</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="J40" s="5" t="s">
         <v>13</v>
@@ -2580,25 +2583,25 @@
         <v>46</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D41" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="E41" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="E41" s="7" t="s">
-        <v>219</v>
-      </c>
       <c r="F41" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="J41" s="5" t="s">
         <v>13</v>
@@ -2615,31 +2618,31 @@
     </row>
     <row r="42" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="J42" s="5" t="s">
         <v>13</v>
@@ -2656,31 +2659,31 @@
     </row>
     <row r="43" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C43" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="I43" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="J43" s="5" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Update test plan and test cases
</commit_message>
<xml_diff>
--- a/02_Manual_Testing/Test_Cases.xlsx
+++ b/02_Manual_Testing/Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my things\SQA projects\BookStack Demo WebTesting\BookStackDemo_WebTesting\02_Manual_Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2133069D-370A-4982-B92A-E04B49E20684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A69D72A-3163-48C7-B2E6-AC2009E85EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1746,7 +1746,7 @@
         <v>13</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="L20" s="5" t="s">
         <v>98</v>
@@ -1951,7 +1951,7 @@
         <v>21</v>
       </c>
       <c r="K25" s="5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>98</v>

</xml_diff>